<commit_message>
docs(evals): round7 终裁落地——41 对终值 MAE 0.342/方向 97.6%，rubric v7 四项改动定稿
</commit_message>
<xml_diff>
--- a/evals/judge_calibration/data/judge-sample-round7-blind-v2.xlsx
+++ b/evals/judge_calibration/data/judge-sample-round7-blind-v2.xlsx
@@ -2,35 +2,86 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标注表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'标注表'!$A$1:$F$42</definedName>
+  </definedNames>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color rgb="FF0563C1"/>
+      <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI Emoji"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -42,12 +93,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,10 +111,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -75,9 +127,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -436,12 +496,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
@@ -449,6 +509,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="96" customWidth="1" min="6" max="6"/>
+    <col width="131.5" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,8 +543,13 @@
           <t>material_summary</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="320" customHeight="1">
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes </t>
+        </is>
+      </c>
+    </row>
+    <row r="2" hidden="1" ht="320.1" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -494,8 +560,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -535,7 +605,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="320" customHeight="1">
+    <row r="3" hidden="1" ht="320.1" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -546,8 +616,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -559,8 +633,13 @@
 【bull】论点: 技术面多头排列+零轴上方金叉+RSI未超买，趋势健康仍有空间; 宏观温和通胀+宽松流动性支撑零售资产质量，整体中性偏正面; ROE 13.44%仍大幅领先同业，盈利质量与现金流优异，增长趋缓恰是低位布局窗口; 舆情偏正面：市值重回万亿、换届有序、行业资金面回暖，四维信号共振 各位评委，从四位分析师的交叉验证来看，招商银行是当前市场中确定性与估值性价比兼备的核心标的。第一，技术面多头排列、MACD零轴上方金叉、RSI偏强未超买，说明趋势健康且仍有上行空间，而非顶部信号——技术动能是本轮行情的领先确认。第二，宏观面温和通胀叠加流动性平稳宽松，利率低位虽压制息差，但同时显著支撑零售信贷资产质量，而资产质量正是零售银行的生命线，宏观组合对招行整体中性偏正面。第三，基本面ROE虽缓慢下行至13.44%，但这一水平仍大幅领先股份行同业，盈利质量高、现金流优异，'增长趋缓'不等于'价值衰退'，恰恰是估值低位介入的窗口。第四，舆情面业绩稳健、市值重回万亿、高管换届有序推进，行业资金面回暖，无明显负面舆情集中，市场共识正在向多头汇聚。综合四维信号共振向上，招行的投资价值清晰：以同业最优的盈利质量，买入一个技术趋势确立、宏观顺风、情绪回暖的时点，风险收益比占优。 【bear】论点: ROE 缓慢下行至 13.44%，健康度评分 48.8，基本面增长动能持续减弱; 利率低位对净息差构成长期压力，侵蚀银行核心利润来源; 舆情偏正面意味着利好已被定价，缺乏边际催化剂，预期落空风险高; 技术面多头排列反映历史，不能对冲基本面减速的估值压力 从看空角度看，招商银行当前的投资风险不容忽视。第一，增长引擎明显减速：基本面报告显示 ROE 已缓慢下行至 13.44%，健康度评分仅 48.8，分析师明确提示'增长趋缓'，说明高盈利质量正被规模扩张放缓和息差收窄侵蚀。第二，宏观面的'中性偏正面'判断过于乐观——利率低位确实支撑资产质量，但对银行而言净息差是核心利润来源，息差持续承压意味着未来营收和利润增速大概率继续下台阶，这是零售银行无法回避的结构性压力。第三，技术面的多头排列只反映历史走势，RSI 偏强但 MACD 已在零轴上方运行一段时间，短期动能'健康'恰恰可能对应阶段性高位，技术信号无法对冲基本面增速放缓的估值压力。第四，舆情面偏正面往往意味着预期已较充分反映在股价中——市值重回万亿、行业资金回暖等利好已被市场定价，缺乏新的边际催化剂，一旦业绩增速低于预期，情绪反转的风险较大。综上，稳健不等于便宜，增长趋缓叠加息差压力，当前价格未必提供足够的安全边际。 【bull】论点: ROE 13.44%仍居股份行第一梯队，评分48.8是静态输出，利润含金量优于悲观暗示; 息差压力全行业共有，招行负债成本优势使其成为相对受益者，资产质量支撑被低估; 资金回暖是进行时，换届落地是未兑现催化，万亿市值是情绪修复起点; 技术趋势是基本面价格化确认，金叉未超买表明趋势处于中段 针对空方四个论点逐条回应。回应对方①：ROE 13.44%看似'下行'，但请评委注意比较基准——这在股份行乃至全行业仍属第一梯队，健康度评分48.8是量化模型的静态输出，分析师同时强调'盈利质量高、现金流优异'，招行的利润含金量（拨备覆盖、不良生成）远优于评分所暗示的悲观图景；ROE缓降但绝对水平领先，恰说明这是行业周期底部而非个体衰退。回应对方②：息差压力我方从未否认，但宏观报告的结论是'整体中性偏正面'——利率低位对零售资产质量的支撑作用被空方系统性低估。银行估值的核心变量从来不是息差的短期弹性，而是资产质量的确定性；招行零售客群优质，不良风险可控，息差收窄是全行业共同面对的环境，而招行凭借负债端成本优势，在同业中息差韧性最强，是压力环境下相对受益者。回应对方③：'利好已被定价'缺乏证据支撑——舆情面显示'行业资金面回暖'，资金流入是正在进行时而非完成时；高管换届有序推进本身即是尚未完全落地的正面催化，且若如空方所言预期已充分，市值刚重回万亿的位置恰是情绪修复的起点而非终点。回应对方④：技术面多头排列不是'反映历史'，而是市场参与者用真金白银投票的结果，是基本面信息的价格化确认；MACD零轴上方金叉+RSI未超买表明趋势处于中段而非顶部，趋势确立恰恰降低了追高风险。综上，空方所有论点均建立在'线性外推悲观情景'之上，而四维信号共振向上的现实摆在这里：用合理估值买入同业最优盈利质量的银行股，安全边际由资产质量和低预期提供，风险收益比明确占优。 【bear】论点: 技术多头排列为滞后信号，无法对冲ROE下行带来的估值压力; 息差压力是结构性利空，资产质量支撑是周期性利好，宏观账算不平; 增长趋缓谈'低位布局'缺乏拐点确认，存在价值陷阱风险; 舆情利好已充分定价，缺乏边际催化剂，业绩不及预期将引发情绪反转 对方在R1中声称招行是'确定性与估值性价比兼备'的核心标的，四维信号共振向上，我认为这一结论存在三处过度乐观。第一，回应对方①——技术面多头排列与零轴上方金叉确实是趋势确认，但技术报告自己也承认RSI已偏强、MACD在零轴上方运行一段时间，趋势确认信号出现在价格已上行之后，本质是滞后指标；在ROE下行通道中，技术动能无法支撑估值中枢上移，一旦业绩增速下台阶，多头排列可能快速瓦解。第二，回应对方②——对方将宏观定性为'中性偏正面'，却回避了关键权衡：利率低位对净息差的压力是持续性、结构性的，而资产质量的支撑是周期性的。宏观报告明确指出息差承压是银行核心利润来源受侵蚀，以周期性利好对冲结构性利空，这个账算不平。第三，回应对方③——'增长趋缓恰是低位布局窗口'是典型的价值陷阱逻辑：健康度评分仅48.8已提示基本面质量存在隐忧，ROE从高位缓慢下行尚未看到拐点确认，在下行趋势中谈'低位'缺乏依据，13.44%领先同业只能说明行业整体承压，不能证明招行自身动能修复。第四，回应对方④——市值重回万亿、资金面回暖等利好已被充分定价，缺乏边际催化剂，一旦中报增速低于市场预期，情绪面将由正转负，放大股价回撤。结论：对方将'稳健'直接等同于'值得买入'，忽视了增长动能减弱与息差压力带来的估值持续压缩风险，当前风险收益比未必占优。 交锋覆盖: bull 论点被回应 4/4；bear 论点被回应 4/4</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="320" customHeight="1">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>个别论点未引数据（bull②/bear②）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" hidden="1" ht="320.1" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -571,8 +650,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -612,8 +695,18 @@
 </t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="320" customHeight="1">
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>1.针对macro的引用解析不客观："利率低位支撑零售资产质量" —— 只能推出"有托底作用、但力度存疑"，不能推出"支撑"这个偏积极的表述；真正支撑资产质量论断还需要不良率、居民收入/就业类数据。需要打补丁的部分：「利率低位支撑零售资产质量」⚠️
+这句话方向上有道理，但从你的数据出发，论证是单向且不完整的：
+利率低位 → 减轻借款人付息负担 → 零售客户（按揭、信用卡、消费贷）违约率承压下降。这条传导链成立，但它是一个"机制推断"，你的论据里没有任何直接关于资产质量的数据（如不良率、关注类贷款、居民收入/失业率）。
+反向压力被忽略了：8月制造业 PMI 49.8、非制造业 49.0，双双在荣枯线以下，M1（4.0%）显著低于 M2（7.7%）、剪刀差 3.7 个百分点说明资金活化不足、企业投资和居民消费意愿偏弱。经济景气度收缩对零售资产质量是负面信号——就业和收入预期才是零售信用风险的根因。PMI 跌破荣枯线恰恰是零售资产质量最需要警惕的先行指标。
+所以对招行这类零售占比高的银行，准确的说法应该是："低利率环境对零售资产质量有托底作用，但景气度走弱构成对冲，资产质量压力中性，需观察 PMI 能否回到荣枯线上方。"
+2.针对[risk_conservative] "激进方紧止损（36.5-37.0）"未能在conservative中找到相同数值的引用。引用9数字与conservative原文(37.5)不一致——但conservative系误转，激进方原话即36.5-37.0；按「对全材料为真」判有出处。数字在此仅为指认、不承重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="320.1" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -624,8 +717,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/1caf1f7bd58a200e532cf521a8a5d9ec</t>
@@ -656,7 +753,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="320" customHeight="1">
+    <row r="6" hidden="1" ht="320.1" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>4758fdb7d62276eedf26a46d3743e010</t>
@@ -667,8 +764,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/4758fdb7d62276eedf26a46d3743e010</t>
@@ -709,7 +810,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="320" customHeight="1">
+    <row r="7" hidden="1" ht="320.1" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>4758fdb7d62276eedf26a46d3743e010</t>
@@ -720,8 +821,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/4758fdb7d62276eedf26a46d3743e010</t>
@@ -733,8 +838,13 @@
 【bull】论点: KDJ深度超卖对应历史底部区域，技术面利空已被充分定价; 宽松流动性环境（低通胀、低LPR）+稳增长政策预期利好半导体国产替代主线; 收入利润重回增长确认周期拐点，重资本开支是产能护城河的战略投资而非价值毁灭; 个股舆情利空真空，向上催化弹性大 综合四份分析师报告，我认为当前正是布局中芯国际的逆向时机。第一，技术面报告明确指出KDJ深度超卖，历史上超卖极值往往对应阶段性底部区域，且均线空头排列、MACD死叉已是市场共识并被充分定价，边际下行空间有限。第二，宏观面并非全面恶化：低通胀与LPR低位意味着流动性环境宽松，政策工具箱充足，PMI虽跌破荣枯线但往往倒逼稳增长政策加码，半导体作为国产替代核心赛道将优先受益。第三，也是最重要的，基本面报告确认公司'收入利润重回增长、财务结构稳健'——周期拐点已经确立。诚然ROE 3.4%、自由现金流-398.7亿元是压制项，但重资本扩张本质是战略卡位：在成熟制程供不应求、地缘政治驱动的国产化大潮下，当前的资本开支正在转化为未来的产能护城河与市场份额。半导体是典型强周期行业，底部扩张、顶部收获是龙头标准打法，台积电历史已多次验证。健康度评分44分反映的是当期回报被压制的静态状况，而非成长逻辑的破坏。第四，舆情面无个股负面新闻恰恰说明利空真空，一旦出现业绩超预期或行业催化，向上弹性大。综合来看，'周期修复+国产替代+超卖点位'三重共振，当前估值提供了中长期布局的风险收益比。 【bear】论点: 技术面中期下行趋势明确：均线空头排列、MACD零轴下死叉，短期反弹动能不足; 健康度评分44分处预警区间，ROE仅3.4%、自由现金流-398.7亿元，重资本扩张严重侵蚀股东回报; 宏观PMI跌破荣枯线、M2增速放缓、资金活化不足，需求端承压压制代工稼动率与价格; 舆情面无个股催化事件，缺乏情绪支撑，而市场已对国产替代提前定价 各位，从四份分析师报告看，看空中芯国际的理由是充分且具体的。第一，技术面明确处于中期下行趋势：均线空头排列、MACD在零轴下方死叉，说明卖压主导；KDJ深度超卖虽常被解读为反弹信号，但在下行趋势中超卖可以钝化，报告自己也承认「短期反弹动能不足」。第二，基本面虽收入利润重回增长，但健康度评分仅44分、处于预警区间，这是最直接的风险信号：ROE仅3.4%，自由现金流高达-398.7亿元，说明增长是靠巨额资本开支堆出来的，股东回报被持续稀释。在半导体行业整体盈利压力下，中芯的扩产可能加剧供过于求，折旧进一步吞噬利润。第三，宏观面PMI跌破荣枯线、M2增速放缓、资金活化不足，需求端承压直接压制晶圆代工的稼动率与价格，低利率环境救不了需求。第四，舆情面近10条新闻无一条涉及个股，事件驱动催化剂缺位，缺乏情绪与资金面的正面支撑。综合来看：估值层面市场对「国产替代」的乐观预期已提前定价，而ROE 3.4%的现实回报远不能支撑，技术趋势、需求疲弱、现金流红灯三重压力叠加，下行风险显著大于上行空间。 【bull】论点: 趋势指标滞后、超卖指标先行，在基本面拐点确立背景下深度超卖是底部特征而非下跌延续; 以台积电历史为例，扩产期低ROE是逆周期投资标准打法，折旧高峰后盈利弹性将释放; PMI破荣枯线触发稳增长政策加码，且国产替代驱动来自供应链安全结构性力量，宏观敏感度低; 空方'无催化'与'已充分定价'论述自相矛盾，超卖+舆情真空说明悲观预期已出清 针对空方四个论点，我逐条回应。回应对方①：技术面报告的完整表述是'中期下行趋势'与'KDJ深度超卖'并存，这正是典型的底部特征组合而非持续下跌信号——趋势指标（均线、MACD）是滞后指标，反映的是已发生的跌幅；而超卖指标是先行指标，反映的是卖压耗尽。空方说超卖会'钝化'，但钝化的前提是基本面持续恶化，而基本面报告确认'收入利润重回增长'，周期拐点已现，超卖钝化的条件并不成立。用滞后指标否定先行指标，是空方技术分析的逻辑漏洞。回应对方②：ROE 3.4%和自由现金流-398.7亿元确实是事实，但空方犯了对强周期成长股用成熟期估值框架的错误。台积电在2009-2012年扩产高峰期ROE同样一度跌至个位数，正是那轮逆周期扩张奠定了其后十年的代工霸主地位。中芯当前折旧高峰恰是产能爬坡期，收入重回增长说明新增产能正被需求消化；健康度评分44分度量的是静态财务健康，而非动态战略价值——地缘政治下国产替代产能的稀缺性溢价无法被DCF模型捕捉。回应对方③：PMI跌破荣枯线恰是政策加码的触发条件，宏观报告明确'宏观环境对中芯国际中性偏宽松'，低通胀+低LPR给了政策充足空间；且半导体国产替代逻辑对宏观景气度的敏感度远低于周期品，其驱动来自供应链安全这一结构性力量。回应对方④：空方一边说'无个股催化'，一边说'国产替代已提前定价'，二者自相矛盾——若已充分定价，为何技术面还能深度超卖？舆情真空+超卖极值恰恰说明悲观预期已出清，预期差向上。综上，空方用静态财务指标和滞后技术指标否定一个周期拐点已确立、战略卡位明确的国产龙头，恰恰是最佳的中长期布局窗口。 【bear】论点: 趋势指标（均线空头、MACD零轴下死叉）优先于震荡指标，下行趋势中超卖可钝化，「利空充分定价」缺乏依据; 宽松流动性无法对冲PMI跌破荣枯线的需求疲软，「政策加码」是未发生的假设，代工稼动率与价格由需求决定; ROE 3.4%、自由现金流-398.7亿元、健康度44分证明扩产尚未产生回报，成熟制程缺乏台积电式定价权，类比不成立; 舆情无个股催化剂是双向真空，技术下行趋势中更可能阴跌，「利空真空=向上弹性」是把信息不足误读为利多 我逐条回应多方上一轮的论点。回应对方①：多方称「KDJ深度超卖对应历史底部、利空已被充分定价」，这是典型的逆势抄底逻辑误区。技术面报告的结论是中期下行趋势——均线空头排列、MACD零轴下方死叉，趋势指标优先级高于震荡指标。在空头排列的下行通道中，超卖可以长期钝化，「充分定价」是主观臆断而非报告结论，报告原文明确「短期反弹动能不足」。用震荡指标否认趋势指标，是拿弱信号反驳强信号。回应对方②：多方将低LPR、低通胀解读为利好，但宏观报告的核心结论是「中性偏宽松但需求端承压」。宽松的流动性救不了PMI跌破荣枯线的实体经济需求——半导体代工的营收取决于下游稼动率与价格，而非利率水平。且「PMI倒逼政策加码」是尚未发生的假设，用预期中的政策对冲已确认的需求疲软，逻辑上不成立。回应对方③：这是多方最核心也最脆弱的论点。「重资本开支是产能护城河」需要两个前提：一是需求确定，二是折旧后能盈利。当前PMI弱势下扩产，恰恰可能加剧供过于求——健康度评分44分、ROE仅3.4%、自由现金流-398.7亿元，三项硬数据证明当前开支尚未转化为回报，反而持续吞噬现金流。台积电在周期底部扩张成功，靠的是技术代差带来的定价权；中芯聚焦的成熟制程竞争激烈、价格弹性弱，不能简单类比。回应对方④：多方称「无负面新闻=利空真空、向上弹性大」，但舆情报告的结论是「判断依据不足、中性偏谨慎」。无正面个股催化剂同样是事实——缺乏事件驱动时，在技术下行趋势中股价更可能随板块资金面阴跌，而非凭空反弹。结论：多方四个论点中，两个引用了报告未作出的乐观推断（底部定价、政策加码），一个用不恰当的类比（台积电）掩盖ROE 3.4%与-398.7亿自由现金流的现实，一个把信息真空误读为利多。基本面预警区间+技术下行趋势+需求承压的三角压制未变，维持看空。 交锋覆盖: bull 论点被回应 4/4；bear 论点被回应 4/4</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="320" customHeight="1">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>个别论点未引数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" hidden="1" ht="320.1" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>4758fdb7d62276eedf26a46d3743e010</t>
@@ -745,8 +855,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/4758fdb7d62276eedf26a46d3743e010</t>
@@ -788,7 +902,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="320" customHeight="1">
+    <row r="9" ht="320.1" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>4758fdb7d62276eedf26a46d3743e010</t>
@@ -799,8 +913,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/4758fdb7d62276eedf26a46d3743e010</t>
@@ -832,7 +950,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="320" customHeight="1">
+    <row r="10" hidden="1" ht="320.1" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>5a059d88512224132b6eff3b02d6226d</t>
@@ -843,8 +961,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5a059d88512224132b6eff3b02d6226d</t>
@@ -889,7 +1011,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="320" customHeight="1">
+    <row r="11" hidden="1" ht="320.1" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>5a059d88512224132b6eff3b02d6226d</t>
@@ -900,8 +1022,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5a059d88512224132b6eff3b02d6226d</t>
@@ -913,8 +1039,13 @@
 【bull】论点: 经营现金流/净利润降至0.75主因票据结算与渠道投放节奏导致的回款滞后，而非终端需求恶化; 经营现金流绝对规模仍超千亿，货币资金超1500亿，负债率低于20%，流动性风险可忽略; 留存现金流为负是加大分红回馈股东的主动资本配置，并非造血能力恶化; 2025年营收下滑是控量保价挤渠道泡沫的战略选择，提价与i茅台放量预示回款质量回升; 低利率环境下高股息确定资产吸引力提升，主力资金净流入叠加技术面超跌提供布局机会 从看多角度审视贵州茅台的经营性现金流问题，我认为市场对现金流健康度的担忧存在过度解读。第一，经营现金流/净利润降至0.75确实低于历史均值，但需要指出，茅台2024年同期该比率超过1.0，本轮下滑主因是渠道政策调整——加大了对经销商的票据结算支持及i茅台渠道投放节奏变化，导致回款暂时性滞后，而非销售终端需求塌方；53度飞天茅台批价虽有回落但仍保持明显顺价，渠道利润空间仍在，这决定了回款只是「迟到」而非「消失」。第二，茅台的经营现金流绝对规模依然是A股天花板级别：即便比率降至0.75，年经营现金流净额仍超千亿元，货币资金储备超1500亿，资产负债率长期低于20%，几乎无有息负债，偿债与流动性风险可以忽略。第三，留存现金流为负并非造血能力恶化的信号，而是公司主动加大分红与特别分红力度、回馈股东的体现——对于一家资本开支需求极低（产能扩建投资进度可控）的轻资产商业模式公司，将现金分配给股东恰恰是资本配置效率最优的选择。第四，2025年营收利润罕见下滑是主动控量保价、挤压渠道泡沫的战略性选择，配合提价与i茅台渠道放量（舆情面正面印证），渠道体系更健康后，现金流回款质量有望在2026-2027年回升。第五，宏观流动性充裕、LPR维持低位背景下，无风险利率下行提升茅台这类确定性高股息资产的估值吸引力，主力资金持续净流入正反映长线资金已在利用技术面超跌（KDJ深度超卖）逢低布局。综上，经营性现金流的短期波动是渠道调整期的阵痛，茅台的商业模式（先款后货、预收款蓄水池）决定了其现金流质量在全市场仍属顶级，当前的现金流担忧恰恰提供了低位布局机会。 【bear】论点: 经营现金流/净利润降至0.75，盈利质量明显稀释，回款质量恶化; 留存现金流为负，分红与资本开支需消耗存量资金，财务安全边际被侵蚀; 宏观需求疲弱是趋势性问题，现金流恶化将滞后延续; 提价在需求疲弱下可能加剧渠道压货，进一步恶化经营现金流 从看空角度审视用户最关心的经营性现金流问题：贵州茅台的现金流正在亮起黄灯。第一，经营现金流/净利润比率已从历史通常大于1的水平降至0.75，意味着每1元净利润只有0.75元真金白银流入，盈利质量明显稀释，可能源于渠道回款放缓、票据结算比例上升——这正是终端需求疲弱在报表上的映射。第二，留存现金流已转负，说明经营现金流不足以覆盖资本开支与分红承诺，长期需消耗账面资金或加杠杆维持高分红，这会侵蚀财务安全边际。第三，回应宏观层面的乐观：分析师明确指出低通胀+PMI弱收缩+M1偏低，高端白酒需求端疲弱是趋势性问题而非短期扰动，现金流恶化是需求收缩的滞后结果，后续季度可能进一步走低。第四，回应舆情面的正面解读：资金净流入和提价预期属于情绪驱动，而2026年中报净利润已实际下滑，基本面兑现不及情绪，提价在需求疲弱环境下反而可能加速渠道压货、恶化回款质量。技术面均线全破、MACD零轴下死叉也印证市场对现金流恶化的定价尚未结束，超跌反弹不改下行趋势。 【bull】论点: 现金净利比0.75是票据结算与i茅台回款节奏错位的时点性问题，飞天批价仍顺价证明回款只是迟到而非消失; 超1500亿货币资金+负债率低于20%，留存现金流为负不构成财务安全边际侵蚀，高分红是轻资产模式的最优资本配置; 流动性充裕+低利率提升高股息资产吸引力，行业收缩期份额向茅台集中; 控量保价出清渠道库存后提价与i茅台放量，回款质量2026-2027年有望回升，超跌提供布局窗口 针对看空方对经营性现金流的四点质疑，我逐条回应。回应对方①：对方称现金净利比0.75意味着盈利质量明显稀释，但对方忽略了该指标的分子分母结构——茅台采用先款后货模式，预收款（合同负债）是天然的蓄水池，比率下滑主要是票据结算支持经销商和i茅台渠道回款节奏错位所致，属于渠道调整的会计时点问题，而非终端动销坍塌；53度飞天批价仍稳定顺价，渠道库存去化后回款会重新入表，2024年该比率曾超1.0，证明公司回款能力有充分的历史弹性。回应对方②：对方称留存现金流为负需消耗存量资金、侵蚀财务安全边际，但账面货币资金超1500亿、资产负债率低于20%、几乎无有息负债，即便连续多年维持当前分红强度，存量资金也远未触及安全边界；将资金返还股东对资本开支极低的轻资产模式而言是资本配置效率的提升，而非财务透支。回应对方③：对方引用宏观需求疲弱论证现金流将持续恶化，但宏观报告同时指出流动性充裕、LPR低位，无风险利率下行正提升高股息确定性资产的配置价值，需求端疲弱压制的是渠道情绪而非茅台的品牌定价权，茅台作为高端白酒绝对龙头恰恰是行业收缩期份额向头部集中的受益者。回应对方④：对方称提价会加剧渠道压货、恶化回款，恰恰相反——2025年营收下滑正是主动控量保价、挤压渠道泡沫的结果，在渠道库存出清的基础上提价与i茅台放量，反映的是公司对终端需求的信心而非压货冲动；舆情面主力资金持续净流入也说明长线资金认可提价逻辑。技术面KDJ深度超跌叠加基本面现金流绝对规模仍超千亿，当前更多是情绪宣泄而非价值重估，恰恰提供了布局窗口。 【bear】论点: 票据结算比例上升本身是渠道资金紧张的信号，与营收同步下滑相互印证，并非单纯结算节奏问题; 留存现金流为负使公司陷入『消耗存量资金维持分红』或『削减分红击穿高股息逻辑』的两难，动摇看多方核心估值依据; 2026中报净利润已实际下滑，『渠道修复后现金流回升』尚无任何报表证据，属于纯预期叙事; 资金净流入与股价走弱并存说明抛压更大，技术面趋势偏空未定价结束 逐条回应看多方第一轮论点： 回应对方①：「票据结算与回款滞后论」。看多方将现金流恶化完全归因于渠道政策调整，称回款只是「迟到」。但这一解释回避了核心问题：票据结算比例上升本身就是渠道资金紧张的信号——经销商需要靠票据而非现金打款，说明其资金链承压，而这背后正是终端动销放缓、批价回落压缩渠道利润的结果。若终端需求真的健康，公司无需加大对经销商的票据支持力度。分析师报告明确指出「2025年营收利润罕见下滑」与现金流比率下降同步出现，若只是结算方式问题，营收不应同时下滑。回款「迟到」还是「消失」，取决于渠道能否消化库存，在PMI弱收缩、M1偏低的宏观环境下，我倾向于前者正在向后者的风险演化。 回应对方②：「千亿现金流绝对规模论」。我不否认绝对规模庞大，但用户问的是现金流是否「健康」，比率比绝对值更诚实。0.75的比率对比茅台自身历史水平（通常≥1）是显著的盈利质量稀释，用绝对规模掩盖结构性恶化，是用「大」回避「变差」的问题。 回应对方③：「留存现金流为负是主动分红」。这是本轮最需要拆穿的乐观叙事：分红是刚性的，而经营现金流是波动的。一旦经营现金流继续下滑（宏观需求疲弱下很可能），公司将在「消耗存量资金维持分红」和「削减分红打击股息叙事」之间二选一——后者会直接击穿看多方第五点所依赖的「高股息确定性资产」逻辑。负留存现金流不是问题本身，但它是该逻辑的脆弱点。 回应对方④：「控量保价战略论」。2026年中报净利润已实际下滑（分析师报告明确提示），「渠道更健康后现金流回升」至今没有任何报表证据，纯属预期。在需求端疲弱（宏观分析明确为趋势性而非短期扰动）的背景下，提价反而可能加剧渠道压货、恶化回款——这一点我第一轮已论述，看多方未正面回应。 回应对方⑤：「主力资金净流入+超跌布局」。技术面分析师结论是股价跌破全部短中期均线、MACD零轴下方死叉且绿柱放大，趋势性偏空。资金净流入与股价持续走弱并存，恰恰说明抛压更大。用长线资金「逢低布局」叙事对抗明确的下行趋势，属于情绪驱动而非数据驱动。 结论：看多方的五点论据中，②③是「用静态优势掩盖动态恶化」，①④⑤是「用预期替代已兑现的报表事实」。2025年报与2026中报已经给出的信号是：盈利下滑+现金流比率0.75+留存现金流为负，三者叠加并非巧合，而是需求收缩传导至报表的完整链条。 交锋覆盖: bull 论点被回应 5/5；bear 论点被回应 4/4</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="320" customHeight="1">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>个别论点未引数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" hidden="1" ht="320.1" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>5a059d88512224132b6eff3b02d6226d</t>
@@ -925,8 +1056,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5a059d88512224132b6eff3b02d6226d</t>
@@ -971,8 +1106,13 @@
 </t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="320" customHeight="1">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>理由段「安全性健康、质量边际恶化」可分解至引用4/5+1/2/6（中性方原话），无引用不算缺；但「辩论各方共识」夸大——激进方否认质量恶化，实为中性+保守方立场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="320.1" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>5a059d88512224132b6eff3b02d6226d</t>
@@ -983,8 +1123,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5a059d88512224132b6eff3b02d6226d</t>
@@ -1020,7 +1164,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="320" customHeight="1">
+    <row r="14" hidden="1" ht="320.1" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1031,8 +1175,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1072,7 +1220,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="320" customHeight="1">
+    <row r="15" hidden="1" ht="320.1" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1083,8 +1231,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1097,7 +1249,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="320" customHeight="1">
+    <row r="16" hidden="1" ht="320.1" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1108,8 +1260,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1149,8 +1305,13 @@
 </t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="320" customHeight="1">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>引用6逐字对上（保守R2「用预期对抗事实」）；理由段引号内转述词序反转（「用事实对抗预期」），语义等价、归属正确，仅引号非逐字。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="320.1" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1161,8 +1322,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5e9b09e3eede28f035b76ef977dd1936</t>
@@ -1193,7 +1358,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="247" customHeight="1">
+    <row r="18" ht="246.95" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>5f41a49aabd8857bdea292b001d365ac</t>
@@ -1204,8 +1369,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/5f41a49aabd8857bdea292b001d365ac</t>
@@ -1220,7 +1389,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="320" customHeight="1">
+    <row r="19" ht="320.1" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>78e31ce92121f73ab38a5682185aec3f</t>
@@ -1231,8 +1400,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/78e31ce92121f73ab38a5682185aec3f</t>
@@ -1247,7 +1420,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="221" customHeight="1">
+    <row r="20" ht="221.1" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>7e6bc8bcfb8800604f23f86449aa7b8c</t>
@@ -1258,8 +1431,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/7e6bc8bcfb8800604f23f86449aa7b8c</t>
@@ -1274,7 +1451,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="320" customHeight="1">
+    <row r="21" hidden="1" ht="320.1" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1285,8 +1462,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1330,7 +1511,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="320" customHeight="1">
+    <row r="22" hidden="1" ht="320.1" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1341,8 +1522,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1355,7 +1540,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="320" customHeight="1">
+    <row r="23" hidden="1" ht="320.1" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1366,8 +1551,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1412,7 +1601,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="320" customHeight="1">
+    <row r="24" ht="320.1" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1423,8 +1612,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/8bbe659aa32218050bf4ae7406de3e15</t>
@@ -1459,7 +1652,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="221" customHeight="1">
+    <row r="25" ht="221.1" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>b17190d6d65bb26efb5cbf069a08b482</t>
@@ -1470,8 +1663,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/b17190d6d65bb26efb5cbf069a08b482</t>
@@ -1486,7 +1683,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="320" customHeight="1">
+    <row r="26" hidden="1" ht="320.1" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>ce66d316a93d8f6069686b8e016aa956</t>
@@ -1497,9 +1694,13 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="C26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/ce66d316a93d8f6069686b8e016aa956</t>
         </is>
@@ -1539,7 +1740,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="320" customHeight="1">
+    <row r="27" hidden="1" ht="320.1" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>ce66d316a93d8f6069686b8e016aa956</t>
@@ -1550,8 +1751,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/ce66d316a93d8f6069686b8e016aa956</t>
@@ -1563,8 +1768,13 @@
 【bull】论点: 顶级基本面护城河：ROE 32.5%、毛利率91%+、零有息负债，稀缺商业模式未变; 技术面KDJ超卖+中长期均线支撑+主力资金明显回流，超跌反弹概率大; 低通胀+低利率+流动性宽松环境对估值形成支撑，分析师判断宏观中性略偏多; i茅台直销渠道改革与提价空间构成量价双重支撑 各位投资者，我从看多角度阐述贵州茅台的投资价值。第一，基本面护城河无可撼动：ROE高达32.5%、毛利率91%以上、几乎零有息负债，这是A股极稀缺的商业模式，即使2025年营收利润首次同比下滑，其盈利质量仍远超绝大多数消费股，周期低谷恰是长期资金布局顶级资产的时机。第二，技术面短期均线空头排列看似利空，但KDJ已进入超卖区间，且中长期均线仍构成有效支撑，技术性超跌往往孕育反弹动能，主力资金近期明显回流即为佐证。第三，宏观面低通胀+利率低位+流动性中性偏宽松的环境，对高端白酒的估值分母端形成支撑；分析师结论也明确判断宏观环境'整体中性略偏多'。第四，渠道改革持续推进，i茅台常态化投放提升直销占比、强化终端掌控力，叠加出厂价体系下的潜在提价空间，量价工具箱依然充足。综上，'高质量但成长熄火'恰恰意味着市场已充分定价悲观预期，估值处于消化阶段，当前的回落是长期投资者的黄金窗口。 【bear】论点: 2025年营收利润首次同比下滑，'永续成长'估值逻辑被打破; 健康度评分78.1（谨慎）、GARP未通过，估值与基本面严重背离; 技术面MACD零轴下方死叉、短期均线空头排列，资金持续撤离; 低通胀+弱制造业环境下需求端修复偏弱，终端动销压力向批价传导; i茅台常态化投放挤压渠道利润，批价下行可能引发渠道信心风险 各位评委，我从看空角度揭示贵州茅台当前的投资风险。第一，成长的叙事已经终结——分析师报告明确指出2025年营收利润首次同比下滑，这是茅台上市以来罕见的拐点信号。市场给茅台溢价的核心逻辑从来不是91%的毛利率本身，而是'永续成长'，一旦成长熄火，估值体系需要系统性下修。第二，估值与基本面背离：健康度评分仅78.1（谨慎档），GARP检验未通过，说明当前价格仍按成长股定价，而基本面已呈现价值股甚至周期股特征，戴维斯双杀风险不可忽视。第三，技术面弱势确立：MACD零轴下方死叉、短期均线空头排列，说明机构资金在用脚投票，前期冲高本质是提价预期的一次性透支。第四，宏观环境只是'中性略偏多'，需求端修复偏弱——白酒尤其是高端白酒高度依赖商务宴请和财富效应，在低通胀、弱制造业环境下，终端动销压力会持续向批价传导。第五，对手方最津津乐道的'i茅台常态化投放'实为双刃剑：直营化短期抬升吨价，但常态化放量会挤压渠道利润空间，批价下行一旦失控将引发渠道信心崩塌，这恰恰是最大的隐藏风险。综上，茅台是好公司，但此刻不是好价格，风险收益比不佳。 【bull】论点: 营收下滑是行业周期性被动降速，ROE 32.5%/毛利率91%+/零有息负债证明护城河未损，类比2013-2015年调整后的大幅反弹; 健康度78.1分在A股仍属高分，GARP未通过源于短期增速分母塌陷，估值已在回落中充分消化悲观预期; 空方选择性忽略KDJ超卖、中长期均线支撑与主力资金明显回流，资金是结构切换而非持续撤离; i茅台直销化是渠道利润内部化，公司控量与提价工具箱足以稳定批价体系，'渠道信心崩塌'是缺乏证据的极端推演 感谢空方的系统性质疑，我逐一回应。回应对方①：2025年营收利润首次同比下滑确实是事实，但请注意这是在行业整体深度调整背景下的'被动降速'，而非护城河受损——ROE仍高达32.5%、毛利率91%+、零有息负债，产品稀缺性和品牌定价权分毫未损。周期低谷的收入下滑与'永续成长逻辑被打破'是两回事，历史上茅台在2013-2015年塑化剂+限制三公消费时期同样下滑，随后迎来数倍涨幅，把周期性波动误读为结构性终结，恰是市场过度悲观的来源。回应对方②：健康度评分78.1确实落在'谨慎'档，但78分在白酒乃至全A股仍属高分区间，GARP未通过更多反映的是短期增速分母塌陷，而非资产质量恶化；当前估值已在回落中大幅消化，'估值与基本面严重背离'的表述言过其实。回应对方③：MACD零轴下方死叉、短期均线空头排列我也承认，但空方选择性忽略了同一份技术面报告中的KDJ超卖信号与中长期均线仍构成支撑，且情绪面报告明确指出主力资金近期明显回流——资金并未'持续撤离'，而是短线资金出逃、中长线资金承接的结构切换。回应对方④：需求端修复偏弱属实，但低利率+流动性中性偏宽松的宏观组合对估值分母端是实打实的支撑，分析师结论仍是'整体中性略偏多'而非偏空；且一旦需求边际改善，茅台是弹性最大的品种之一。回应对方⑤：关于i茅台挤压渠道利润、批价失控风险——直销占比提升本质是把渠道利润内部化，即使批价阶段性承压，公司通过控量、提价工具箱完全可以调节供需平衡，历史上茅台从未失去对价格体系的掌控力；把'常态化投放'直接等同于'渠道信心崩塌'，是缺乏中间证据的极端推演。综上，空方描绘的是'戴维斯双杀'的尾部情景，但数据指向的是'高质量资产+悲观预期充分定价'的现实，风险收益比正在向多头倾斜。 【bear】论点: 首次营收利润下滑+现金流质量回落是商业模式边际弱化信号，非普通周期低谷; KDJ超卖在下跌趋势中可钝化，MACD死叉+均线空头主导趋势方向; 宏观报告明确'需求端修复偏弱压制弹性'，分子恶化压倒分母支撑; i茅台常态化投放挤压渠道利润，批价下行威胁品牌价值与提价逻辑; GARP未通过，估值仍按成长股定价，下修空间大 回应对方①：对手承认2025年营收利润首次同比下滑，却轻描淡写为'周期低谷'。但请注意，这是茅台上市以来首次年度下滑，且分析师健康度评分降至78.1（谨慎档）、现金流质量回落，这不是普通周期波动，而是商业模式边际弱化的信号——当渠道库存高企、批价倒挂时，即便ROE仍达32.5%，其可持续性正遭受历史性考验。用'ROE绝对值高'论证安全边际，回避了'趋势向下'这一关键事实。回应对方②：KDJ超卖在下跌趋势中只是超卖可以更超卖，MACD零轴下方死叉与短期均线空头排列才是趋势的主导信号；所谓'主力资金回流'规模有限，无法对冲机构在高位累积的抛压，技术性反弹恰恰是出货窗口而非趋势反转。回应对方③：对手引用宏观'中性略偏多'，却刻意忽略了同一份报告中最关键的半句——'需求端修复偏弱压制弹性'。分母端（利率）的支撑是全局性的，不构成茅台的相对优势；而分子端（需求）的疲弱却是茅台的专属压力。高端白酒依赖商务宴请与财富效应，低通胀+弱制造业环境下，分子恶化将压倒分母利好。回应对方④：对手宣称i茅台构成'量价双重支撑'，但常态化投放的本质是以渠道利润为代价换取报表收入——批价持续阴跌正说明终端承接力不足，一旦批价击穿渠道盈亏平衡线，抛售踩踏将反噬品牌价值与提价逻辑。叠加GARP检验未通过，当前价格仍按成长股定价，估值下修空间显著。结论：好公司≠好价格，在成长叙事证伪、估值消化未完成的阶段，左侧接刀风险远大于机会。 交锋覆盖: bull 论点被回应 4/4；bear 论点被回应 5/5</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="320" customHeight="1">
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>个别论点未引数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" hidden="1" ht="320.1" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>ce66d316a93d8f6069686b8e016aa956</t>
@@ -1575,8 +1785,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/ce66d316a93d8f6069686b8e016aa956</t>
@@ -1618,7 +1832,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="320" customHeight="1">
+    <row r="29" ht="320.1" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>ce66d316a93d8f6069686b8e016aa956</t>
@@ -1629,8 +1843,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/ce66d316a93d8f6069686b8e016aa956</t>
@@ -1673,8 +1891,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/cfe8ca0c8eb1530eb9ad086deaf159bb</t>
@@ -1689,7 +1911,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="320" customHeight="1">
+    <row r="31" hidden="1" ht="320.1" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>d477972f89d24a11593ea9c84c4babb6</t>
@@ -1700,8 +1922,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d477972f89d24a11593ea9c84c4babb6</t>
@@ -1746,7 +1972,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="320" customHeight="1">
+    <row r="32" hidden="1" ht="320.1" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>d477972f89d24a11593ea9c84c4babb6</t>
@@ -1757,8 +1983,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d477972f89d24a11593ea9c84c4babb6</t>
@@ -1771,7 +2001,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="320" customHeight="1">
+    <row r="33" hidden="1" ht="320.1" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>d477972f89d24a11593ea9c84c4babb6</t>
@@ -1782,8 +2012,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d477972f89d24a11593ea9c84c4babb6</t>
@@ -1829,7 +2063,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="320" customHeight="1">
+    <row r="34" ht="320.1" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>d477972f89d24a11593ea9c84c4babb6</t>
@@ -1840,8 +2074,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d477972f89d24a11593ea9c84c4babb6</t>
@@ -1877,7 +2115,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="320" customHeight="1">
+    <row r="35" hidden="1" ht="320.1" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>d7e48a92801a3349142de115eafb389f</t>
@@ -1888,8 +2126,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d7e48a92801a3349142de115eafb389f</t>
@@ -1931,7 +2173,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="320" customHeight="1">
+    <row r="36" hidden="1" ht="320.1" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>d7e48a92801a3349142de115eafb389f</t>
@@ -1942,8 +2184,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d7e48a92801a3349142de115eafb389f</t>
@@ -1955,8 +2201,13 @@
 【bull】论点: 归母净利润高增36%、ROE回升至14%，基本面处于持续修复通道; 低利率环境利好保险产品销售，负债端改善是核心alpha; 中期技术面保持多头排列上行趋势，短期回调提供介入时点; 舆情面正面报道占优，与基本面修复形成正反馈 综合四份分析师报告，我方坚定看多中国平安，理由如下： 第一，基本面持续修复是核心逻辑。归母净利润连续高增，2026年中报净利大增36%，ROE回升至14%，现金流质量优异——这说明公司盈利能力与造血能力同步改善，估值中枢有上移基础。净利润36%的高增长在金融板块中属于稀缺的高弹性，理应享受估值溢价。 第二，宏观环境对保险主业形成实质利好。报告明确指出，低利率环境虽然短期压制新配资产收益率，但'利好保险产品销售与股市风险偏好'。储蓄型保险产品在存款利率、理财收益率下行的背景下相对吸引力显著提升，负债端改善是保险公司最核心的alpha来源，这一利好被市场低估。 第三，舆情面正面占优。净利大增36%驱动正面报道占优，市场情绪与基本面形成正反馈，机构定价正在向修复逻辑靠拢。 第四，技术面短期回调不改中期格局。报告指出中期保持'多头排列的上行趋势'，MACD死叉与KDJ回落只是高位回调整理，恰恰为投资者提供了更优的介入时点，而非趋势逆转信号。 综上，负债端受益于低利率环境、盈利端高增长兑现、中期技术趋势完好，短期回调是布局良机，我方坚定看多。 【bear】论点: MACD死叉与KDJ回落显示短期高位回调，入场时点风险大; 低利率持续压制新配资产收益率，利差损风险长期侵蚀利润; 健康度评分52.1分处警示区间，季度业绩波动大，36%净利高增可持续性存疑; 机构减持叠加寿险代理人持续收缩，资金撤离且核心渠道产能基础萎缩 从看空角度审视中国平安，当前时点的风险不容忽视。第一，技术面已发出明确调整信号：尽管中期维持多头排列，但MACD死叉与KDJ回落表明短期动能衰竭，股价处于高位回调整理阶段，此时入场面临回调风险，历史经验显示高位死叉往往对应数周的调整周期。第二，低利率环境的压制被低估：宏观报告明确指出低利率压制新配资产收益率，平安作为资产规模超十万亿的险资巨头，存量资产到期再配置时收益率持续下移，利差损风险将长期侵蚀利润，这是比短期利润增长更本质的隐患。第三，健康度评分仅52.1分、处于'警示'区间，且季度业绩波动大，说明盈利修复的可持续性存疑，36%的净利高增可能包含投资收益波动等一次性因素，不宜线性外推。第四，资金与渠道双收缩：机构减持叠加寿险代理人队伍持续缩减，前者代表聪明钱撤离，后者意味着核心渠道的产能基础在萎缩，新业务价值增长缺乏支撑。综上，短期技术调整、长期利差损、结构警示与资金撤离四重压力叠加，看空风险显著。 【bull】论点: 中期多头排列趋势优先于短期技术信号，高位死叉多为整理而非反转; 低利率下负债成本同步下行，负债端销售改善是核心alpha，36%净利增长本身就是利差改善证据; 健康度评分52.1分的警示源自保险业天然高杠杆的结构性特征，评分框架对金融股失真; 机构减持被过度解读，舆情整体正面占优，代理人收缩是主动清虚转型、人均产能提升利好新业务价值率 逐条回应对方R1论点，我方认为空方结论站不住脚： 回应对方①：MACD死叉与KDJ回落确实提示短期调整，但报告原文明确界定为'高位回调整理'而非趋势逆转，且中期'多头排列的上行趋势'完好。技术分析的基本原则是中期趋势优先于短期信号，历史经验同样显示上升趋势中的高位死叉多为洗盘而非反转。回调提供的是更优的安全边际，而非风险警报。 回应对方②：低利率压新配资产收益率是事实，但对方忽略了保险的商业模式本质——资产与负债是联动的。宏观报告明确指出低利率'利好保险产品销售'，负债成本随预定利率下调同步下行，利差损的算术题对方只算了一半。负债端改善才是保险公司最核心的alpha，36%的净利高增本身就是利差改善的证据，而非利差损的证据。 回应对方③：健康度评分52.1分的'警示'主要源自'高负债率与低净利率'，而报告原文明确指出这是'保险业结构性特征'——保险公司天然高杠杆经营，用一般行业框架评分对金融股失真，不构成有效的看空依据。至于季度业绩波动，36%的中报净利增速与ROE回升至14%的方向一致，基本面报告的结论是'持续修复通道'，而非不可持续。 回应对方④：机构减持与代理人收缩确是隐忧，但对方过度解读。舆情报告的整体判断是'正面报道占优'，净利大增36%驱动市场情绪与基本面正反馈，主流定价方向仍是修复逻辑。代理人收缩是全行业主动清虚的转型过程，人均产能提升恰恰是新业务价值率改善的前提。 综上，对方的四重压力中：技术信号误读中期趋势、利差损忽略负债端联动、健康度评分框架失真、资金渠道收缩被过度放大。基本面修复+负债端alpha+中期趋势完好的看多逻辑依然成立，短期回调即布局窗口。 【bear】论点: 健康度评分52.1分警示区间+季度业绩波动大，36%净利高增或为投资收益一次性弹性，不可线性外推; 多头选择性引用宏观报告，回避低利率压制新配资产收益率与利差损这一更本质的长期风险; 高位MACD死叉动能衰竭，无企稳证据前称'介入时点'属逆势接刀; 机构减持与代理人收缩两个负面硬数据被多头完全忽略，情绪正反馈随时可逆转 针对多头R1的四个论点，我方逐条反驳： 回应对方①：多头称净利大增36%、ROE回升至14%即处于'持续修复通道'，但基本面报告明确给出健康度评分仅52.1分、处于'警示'区间，且季度业绩波动大。36%的高增很可能是投资收益波动驱动的弹性而非可持续的经营性增长——两者天壤之别，把一次性弹性当作'稀缺高弹性'给予估值溢价，是典型的线性外推错误。ROE回升至14%也仅是修复到行业中等水平，谈不上支撑估值中枢上移。 回应对方②：多头将低利率简化为'利好负债端销售'，刻意回避了报告的前半句——'低利率短期压制新配资产收益率'。对平安这样的险资巨头，资产端是十万亿级盘子，利率每下移一点，到期再配置的利差损就扩大一分。储蓄险好卖的前提是公司能持续兑付有吸引力的预定利率，一旦利差损侵蚀资本，负债端优势反而是加速失血的速度。多头只取宏观报告中对自己有利的半句，属于选择性引用。 回应对方③：多头称MACD死叉、KDJ回落'恰恰是介入时点'，这是把调整风险包装成机会。技术报告的原文判断是'短期处于高位回调整理阶段'——高位死叉对应的是动能衰竭，调整深度与时長均不可知，在信号未修复前入场是逆势接刀。多头无法给出任何死叉已企稳的证据，仅凭中期多头排列就断言'不改格局'，依据不足。 回应对方④：正面报道占优恰恰建立在36%净利的单一叙事上，一旦后续季度业绩波动兑现（基本面报告已提示），情绪反噬会同样剧烈。而机构减持与寿险代理人持续收缩这两个硬数据被多头完全忽略——聪明钱在用脚投票，核心渠道产能基础在萎缩，正反馈随时可能逆转为负反馈。 综上，多头四个论点均存在选择性引用或过度外推，风险未被定价，我方维持看空。 交锋覆盖: bull 论点被回应 4/4；bear 论点被回应 4/4</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="320" customHeight="1">
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>个别论点未引数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" hidden="1" ht="320.1" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>d7e48a92801a3349142de115eafb389f</t>
@@ -1967,8 +2218,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d7e48a92801a3349142de115eafb389f</t>
@@ -2011,7 +2266,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="320" customHeight="1">
+    <row r="38" ht="320.1" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>d7e48a92801a3349142de115eafb389f</t>
@@ -2022,8 +2277,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/d7e48a92801a3349142de115eafb389f</t>
@@ -2056,7 +2315,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="320" customHeight="1">
+    <row r="39" hidden="1" ht="320.1" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>e6816ca8a182b602b512868b36411269</t>
@@ -2067,8 +2326,12 @@
           <t>consistency</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/e6816ca8a182b602b512868b36411269</t>
@@ -2111,7 +2374,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="320" customHeight="1">
+    <row r="40" hidden="1" ht="320.1" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>e6816ca8a182b602b512868b36411269</t>
@@ -2122,8 +2385,12 @@
           <t>debate_quality</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/e6816ca8a182b602b512868b36411269</t>
@@ -2135,8 +2402,13 @@
 【bull】论点: 中期上行趋势未变，短线指标回落仅是技术性回踩，反而提供更佳买点; 现金流质量高+中报净利润小幅增长，体现行业承压期的经营韧性; 机构减持与舆情逆风带来的回调是逆向布局的低估值机会; 宏观利空已充分定价，温和通胀环境无系统性风险 综合四位分析师的判断，我认为当前正是平安银行的战略性布局窗口。第一，技术面分析师确认短期均线多头排列、中期上行趋势延续，这是趋势投资者最重视的信号；MACD柱转负和RSI、KDJ高位回落只是上升趋势中的正常技术性回踩，恰恰为长线资金提供了更好的介入价位，而非趋势反转。第二，宏观面的中性偏空已被市场充分定价——平安银行当前估值处于历史低位区域，PMI走弱与LPR低位虽压制资产端收益率，但同时也压低了负债成本并减少不良生成压力，温和通胀环境意味着不存在系统性风险。第三，基本面分析提到盈利能力回落，但更关键的结论是'现金流质量高'——银行股的核心价值在于资产负债表稳健性和分红能力，而非短期盈利增速；中报净利润仍实现小幅增长，说明在行业普遍承压期公司展现了经营韧性。第四，情绪面整体中性偏正面，机构减持导致的股价回调正是逆向投资的良机。综上，趋势在、现金流稳、估值低、情绪逆风，四者叠加构成了典型的左侧买入机会，风险收益比显著占优。 【bear】论点: 宏观中性偏空：PMI跌破荣枯线、M1-M2剪刀差走阔显示信贷需求疲弱，LPR低位持续压缩净息差; 基本面健康度warning级别且GARP检验不通过，盈利能力持续回落，估值缺乏安全边际; 技术面MACD由正转负、RSI与KDJ高位回落，短线动能衰竭，趋势拐点风险; 机构减持叠加银行板块资金波动，中报仅小幅增长缺乏催化 作为看空方，我认为平安银行当前投资风险大于机会，核心逻辑如下：第一，宏观逆风明确。分析师报告指出PMI已降至荣枯线下方、M2增速放缓、M1-M2剪刀差走阔，这意味着企业活期资金持续沉淀、信贷需求疲弱，银行资产端扩张缺乏动力；同时LPR维持低位，净息差被持续压缩，平安银行以零售信贷见长，在居民收入预期未改善背景下，零售资产质量与定价能力双重承压。第二，基本面健康度已亮黄灯。分析师给出的健康度评级为warning级别，且GARP估值检验不通过——即当前股价相对增长预期并不便宜，盈利能力持续回落（ROE、ROA下滑）的同时估值缺乏安全边际，这不是'便宜的好资产'，而是'不便宜的弱资产'。第三，技术面短线动能衰竭。MACD柱状图刚由正转负、RSI与KDJ高位回落，短期均线虽多头排列但属于滞后指标，动能指标率先转弱往往预示趋势拐点临近，追高面临回调风险。第四，资金与情绪面存在隐忧。舆情虽中性偏正面，但机构减持信号明确，银行板块资金波动加剧，中报净利润仅'小幅增长'缺乏超预期催化，难以吸引增量资金。综上，宏观（中性偏空）、基本面（warning+GARP不通过）、技术（动能转弱）、资金（机构减持）四个维度共振向下，建议规避短期风险。 【bull】论点: 宏观利空已被低估值充分定价，LPR低位同时压低负债成本，是双刃剑而非单向利空; GARP框架不适用于以现金流和分红为核心的银行股，现金流质量高才是安全边际来源; 中期上行趋势延续未被撼动，动能指标回落只是正常回踩并提供更佳买点; 机构减持带来的回调是逆向布局机会，低估值+高分红对长线资金具持续吸引力 感谢空方观点，我逐条回应。回应对方①：您引用PMI跌破荣枯线、M1-M2剪刀差走阔论证宏观逆风，但恰恰忽略了同一份宏观报告的完整结论是'中性偏空'而非系统性看空——温和通胀意味着无滞胀风险，LPR低位固然压缩资产端收益率，但同时降低了负债成本并稳定了资产质量预期，这是双刃剑而非单向利空。且我方R1已指出，这些宏观利空在当前历史低位估值中已被充分定价，边际恶化的空间有限、边际改善（如政策宽松加码、M2企稳）反而是期权。回应对方②：您将'warning级别+GARP不通过'等同于'不便宜的弱资产'，这是对银行股估值框架的误用。银行业负债率与资产周转指标偏弱是行业常态（分析师报告明确说明），GARP检验以增长为核心，天然不适用于以资产负债表稳健性和分红能力为核心价值的银行股；而报告中最被您淡化的事实是'现金流质量高'——这恰恰是银行股安全边际的真正来源，中报净利润在行业普遍承压期仍实现小幅正增长，证明经营韧性而非'弱资产'。回应对方③：您说MACD转负预示趋势拐点，但技术分析师的原始结论是'中期上行趋势延续'、'短期均线多头排列'，动能指标的高位回落在一轮上涨后极为常见，将滞后确认的均线体系仍为多头排列定性为'拐点风险'缺乏数据支撑；退一步说，即便短线回踩，对我方R1所论证的左侧布局逻辑反而是更优的买点而非卖点。回应对方④：机构减持确是事实，但情绪面分析师的整体定性是'中性偏正面'，减持带来的波动恰是逆向资金的筹码来源；中报小幅增长虽非强催化，但在银行板块整体承压背景下已属稳健，估值低位+高分红属性（现金流质量高所支撑）对保险、长线配置资金具备持续吸引力，增量资金未必依赖中报催化。综上，空方的四点均建立在'把正常波动放大为趋势反转、把行业属性误判为公司缺陷'之上，而趋势、现金流、估值三大核心支撑未被撼动，风险收益比仍显著偏向多方。 【bear】论点: 领先动能指标转弱先于滞后均线，技术性回踩说法缺乏依据，趋势拐点风险真实存在; 健康度warning+GARP不通过表明估值缺乏安全边际，'低估值机会'实为价值陷阱; 机构减持是对基本面的否定投票，与逆向布局逻辑自相矛盾; PMI走弱与剪刀差走阔是恶化中的增量信息，'利空已充分定价'不成立 针对多头R1的四个论点，我逐条回应：回应对方①——多头称短线指标回落只是'技术性回踩、提供更佳买点'，这是典型的趋势确认偏误。分析师报告明确指出MACD柱状图'刚由正转负'、RSI与KDJ'高位回落'，在多头排列的滞后均线尚未反转之前，领先动能指标已率先转弱，历史上这正是趋势拐点的标准前兆。把风险信号解读为买点，缺乏数据支撑。回应对方②——多头强调'现金流质量高+中报净利润小幅增长体现韧性'，但回避了分析师的核心结论：健康度评分是warning级别、GARP检验不通过。对银行而言，盈利能力持续回落意味着净息差收窄正在侵蚀长期分红能力的根基，'小幅增长'恰恰说明增长动能接近枯竭，谈不上韧性。回应对方③——所谓'机构减持带来的回调是逆向布局机会'存在致命矛盾：如果低估值真是机会，为何专业机构选择减持？机构比散户拥有更完整的不良率、息差前瞻数据，其减持行为本身就是对基本面的否定投票；叠加银行板块资金波动加剧，'低估值'很可能是价值陷阱而非安全边际——GARP不通过正说明这一点。回应对方④——多头称'宏观利空已充分定价'，但PMI刚降至荣枯线下方、M1-M2剪刀差走阔是正在恶化的增量信息而非存量信息，无法被'充分定价'；且LPR低位压缩息差的同时，负债成本下行空间远小于资产端收益下行速度，多头'压低负债成本对冲'的逻辑在存贷结构上不成立。综上，多头四条论点均建立在对利空信号的乐观再解读之上，缺乏数据验证，我维持看空判断。 交锋覆盖: bull 论点被回应 4/4；bear 论点被回应 4/4</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="320" customHeight="1">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>个别论点未引数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" ht="320.1" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>e6816ca8a182b602b512868b36411269</t>
@@ -2147,8 +2419,12 @@
           <t>decision_grounding</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/e6816ca8a182b602b512868b36411269</t>
@@ -2192,7 +2468,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="320" customHeight="1">
+    <row r="42" ht="320.1" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>e6816ca8a182b602b512868b36411269</t>
@@ -2203,8 +2479,12 @@
           <t>report_relevance</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
           <t>http://localhost:3000/project/cmrd9hmlo0006pe0748wbzohn/traces/e6816ca8a182b602b512868b36411269</t>
@@ -2239,6 +2519,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F42">
+    <filterColumn colId="1" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="report_relevance"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -2283,5 +2570,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>